<commit_message>
feat: implement select component and create teacher form with associated services and pages
</commit_message>
<xml_diff>
--- a/Public/Eparchy of Kanjirappally.xlsx
+++ b/Public/Eparchy of Kanjirappally.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LigthSuvara-Web-App\Public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4CBFC3-AD3A-42E0-AD40-6295661FA93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F15A4901-B64B-4339-99B2-AE924D997FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3170,7 +3170,7 @@
         <v>166</v>
       </c>
       <c r="L214">
-        <v>111</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="215" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3184,7 +3184,7 @@
         <v>159</v>
       </c>
       <c r="L215">
-        <v>112</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="216" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3198,7 +3198,7 @@
         <v>161</v>
       </c>
       <c r="L216">
-        <v>113</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="217" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3212,7 +3212,7 @@
         <v>160</v>
       </c>
       <c r="L217">
-        <v>114</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="218" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3226,7 +3226,7 @@
         <v>165</v>
       </c>
       <c r="L218">
-        <v>115</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="219" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3240,7 +3240,7 @@
         <v>168</v>
       </c>
       <c r="L219">
-        <v>116</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="220" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3254,7 +3254,7 @@
         <v>164</v>
       </c>
       <c r="L220">
-        <v>117</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="221" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3268,7 +3268,7 @@
         <v>158</v>
       </c>
       <c r="L221">
-        <v>118</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="225" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3298,7 +3298,7 @@
         <v>175</v>
       </c>
       <c r="L227">
-        <v>121</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="228" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3312,7 +3312,7 @@
         <v>181</v>
       </c>
       <c r="L228">
-        <v>122</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="229" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3326,7 +3326,7 @@
         <v>177</v>
       </c>
       <c r="L229">
-        <v>123</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="230" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3340,7 +3340,7 @@
         <v>178</v>
       </c>
       <c r="L230">
-        <v>124</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="231" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3354,7 +3354,7 @@
         <v>173</v>
       </c>
       <c r="L231">
-        <v>125</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="232" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3368,7 +3368,7 @@
         <v>179</v>
       </c>
       <c r="L232">
-        <v>126</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="233" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3382,7 +3382,7 @@
         <v>176</v>
       </c>
       <c r="L233">
-        <v>127</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="234" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3396,7 +3396,7 @@
         <v>180</v>
       </c>
       <c r="L234">
-        <v>128</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="235" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3410,7 +3410,7 @@
         <v>169</v>
       </c>
       <c r="L235">
-        <v>129</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="241" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3440,7 +3440,7 @@
         <v>234</v>
       </c>
       <c r="L243">
-        <v>131</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="244" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3454,7 +3454,7 @@
         <v>188</v>
       </c>
       <c r="L244">
-        <v>132</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="245" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3468,7 +3468,7 @@
         <v>189</v>
       </c>
       <c r="L245">
-        <v>133</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="246" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3482,7 +3482,7 @@
         <v>193</v>
       </c>
       <c r="L246">
-        <v>134</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="247" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3496,7 +3496,7 @@
         <v>195</v>
       </c>
       <c r="L247">
-        <v>135</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="248" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3510,7 +3510,7 @@
         <v>191</v>
       </c>
       <c r="L248">
-        <v>136</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="249" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3524,7 +3524,7 @@
         <v>186</v>
       </c>
       <c r="L249">
-        <v>137</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="250" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3538,7 +3538,7 @@
         <v>184</v>
       </c>
       <c r="L250">
-        <v>138</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="251" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3552,7 +3552,7 @@
         <v>192</v>
       </c>
       <c r="L251">
-        <v>139</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="252" spans="8:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -3566,7 +3566,7 @@
         <v>170</v>
       </c>
       <c r="L252">
-        <v>1310</v>
+        <v>13010</v>
       </c>
     </row>
   </sheetData>

</xml_diff>